<commit_message>
SBMD-43 test: PEN paketi 2014/02'ye tasindi, log dosyasi repodan cikarildi
- pentest-2014-02-*.xlsx: yil kolonu 2025 kalmisti, hatali-satirlar dosyasinin
  icerigi (PENTEST2502, 2025) hic degismemisti, iki-donem dosyasinda 15 oneki
  vardi. Uc dosya 2014/02 (+2014/03), PENTEST1402-*, tarih 2014 ile yeniden
  uretildi; tutarlar ve il/ilce ayni.
- PEN koleksiyonlari bruno-pentest-2014-02(-basit).json: PENTEST1402, yil=2014;
  @usebruno/schema ile dogrulandi.
- Eski pentest-2025-02-hatali-satirlar.xlsx ve Lokal Test/Loglar.txt (ic ESB
  adresi, sirket VKN'si) kaldirildi; Loglar*.txt ve *.log .gitignore'da.
- Rehber, README, CLAUDE.md, temizlik SQL'i PENTEST1402 / 2014/02'ye guncellendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pen Test/pentest-2014-02-hatali-satirlar.xlsx
+++ b/Pen Test/pentest-2014-02-hatali-satirlar.xlsx
@@ -53,28 +53,28 @@
     <t>vergiPrimTutari</t>
   </si>
   <si>
-    <t>PENTEST2502-90</t>
+    <t>PENTEST1402-90</t>
   </si>
   <si>
     <t>abc</t>
   </si>
   <si>
-    <t>PENTEST2502-91</t>
-  </si>
-  <si>
-    <t>PENTEST2502-92</t>
-  </si>
-  <si>
-    <t>31-02-2025</t>
-  </si>
-  <si>
-    <t>PENTEST2502-93</t>
-  </si>
-  <si>
-    <t>PENTEST2502-94</t>
-  </si>
-  <si>
-    <t>PENTEST2502-9999999999999999999999999</t>
+    <t>PENTEST1402-91</t>
+  </si>
+  <si>
+    <t>PENTEST1402-92</t>
+  </si>
+  <si>
+    <t>31-02-2014</t>
+  </si>
+  <si>
+    <t>PENTEST1402-93</t>
+  </si>
+  <si>
+    <t>PENTEST1402-94</t>
+  </si>
+  <si>
+    <t>PENTEST1402-9999999999999999999999999</t>
   </si>
   <si>
     <t>X&amp;sigortaSirketKodu=999</t>
@@ -86,10 +86,10 @@
     <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
   </si>
   <si>
-    <t>PENTEST2502-95</t>
-  </si>
-  <si>
-    <t>PENTEST2502-96</t>
+    <t>PENTEST1402-95</t>
+  </si>
+  <si>
+    <t>PENTEST1402-96</t>
   </si>
 </sst>
 </file>
@@ -211,10 +211,10 @@
         <v>2320.0</v>
       </c>
       <c r="E2" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G2" t="s" s="0">
         <v>13</v>
@@ -252,10 +252,10 @@
         <v>2320.0</v>
       </c>
       <c r="E3" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F3" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="H3" t="n" s="2">
         <v>1000.0</v>
@@ -290,10 +290,10 @@
         <v>2320.0</v>
       </c>
       <c r="E4" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F4" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G4" t="s" s="0">
         <v>15</v>
@@ -331,10 +331,10 @@
         <v>2320.0</v>
       </c>
       <c r="E5" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F5" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>16</v>
@@ -375,7 +375,7 @@
         <v>17</v>
       </c>
       <c r="F6" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G6" t="s" s="0">
         <v>18</v>
@@ -413,10 +413,10 @@
         <v>2320.0</v>
       </c>
       <c r="E7" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F7" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G7" t="s" s="0">
         <v>19</v>
@@ -454,10 +454,10 @@
         <v>2320.0</v>
       </c>
       <c r="E8" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F8" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G8" t="s" s="0">
         <v>20</v>
@@ -495,10 +495,10 @@
         <v>2320.0</v>
       </c>
       <c r="E9" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F9" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G9" t="s" s="0">
         <v>21</v>
@@ -536,10 +536,10 @@
         <v>2320.0</v>
       </c>
       <c r="E10" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F10" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G10" t="s" s="0">
         <v>22</v>
@@ -577,10 +577,10 @@
         <v>2320.0</v>
       </c>
       <c r="E11" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F11" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G11" t="s" s="0">
         <v>23</v>
@@ -618,10 +618,10 @@
         <v>2320.0</v>
       </c>
       <c r="E12" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F12" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G12" t="s" s="0">
         <v>24</v>
@@ -659,10 +659,10 @@
         <v>2320.0</v>
       </c>
       <c r="E13" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G13" t="s" s="0">
         <v>13</v>
@@ -700,10 +700,10 @@
         <v>2320.0</v>
       </c>
       <c r="E14" t="n" s="1">
-        <v>45736.0</v>
+        <v>41718.0</v>
       </c>
       <c r="F14" t="n" s="0">
-        <v>2025.0</v>
+        <v>2014.0</v>
       </c>
       <c r="G14" t="s" s="0">
         <v>25</v>

</xml_diff>